<commit_message>
Apply mind-map refinements to ALAGA and lock PH scale
Corrects the repeat-base retention assumption from 0.78 to 0.990 per
month; the original implied ~5% survival at 12 months against a 60%+
benchmark, understating 24-month EBITDA by roughly half and wrongly
disqualifying the US supplier lane on payback. Adds quarterly-default
billing and makes BAI registration the lead brand claim. Records in
the agent manual that the GBP mind map is category research only, not
deployable capital, and carries live project status forward.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkbvziRGAQswinfFBc6fjv
</commit_message>
<xml_diff>
--- a/business/alaga/ALAGA-FLEX-model.xlsx
+++ b/business/alaga/ALAGA-FLEX-model.xlsx
@@ -154,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -215,6 +215,7 @@
     <xf numFmtId="165" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="10" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -305,6 +306,11 @@
     <comment ref="C26" authorId="0" shapeId="0">
       <text>
         <t>Model is more sensitive to this than to FOB cost. Track cohort reorder rate weekly from launch. Operating manual kill criterion: abandon if under 15% by month 4.</t>
+      </text>
+    </comment>
+    <comment ref="C27" authorId="0" shapeId="0">
+      <text>
+        <t>CORRECTED 2 Sep 2026. Previously 0.78/month, which implied only ~5% of the repeat base surviving 12 months — far below observed behaviour. Benchmarks: pet subscription monthly plans churn 18-22% per year, quarterly 11-16%, and subscription pet brands retain 60%+ of customers past month 12. 0.990/month compounds to ~89% annual retention (quarterly billing); 0.982 gives ~80% (monthly billing).</t>
       </text>
     </comment>
   </commentList>
@@ -600,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B39"/>
+  <dimension ref="B2:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -755,7 +761,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>WHAT THE MODEL SAYS AT THESE PLACEHOLDER NUMBERS</t>
         </is>
@@ -764,28 +770,28 @@
     <row r="29">
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Landed cost decides payback, not repeat rate. Tested across both supplier lanes:</t>
+          <t>China lane (FOB $4.00, MOQ 1,000): capital ~PHP 920,000 · payback month 13</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · China lane (FOB $4.00, MOQ 1,000): capital ≈ PHP 918,000 · payback ≈ month 15</t>
+          <t>US lane (FOB $7.00, MOQ 2,500): capital ~PHP 2,091,000 · payback month 21</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · US lane (FOB $7.00, MOQ 2,500): capital ≈ PHP 2,082,000 · payback beyond 24 months</t>
+          <t>Both now clear the 24-30 month screen. The China lane still wins on cash,</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · Varying repeat conversion from 10% to 45% moves China payback only 17 → 15 months.</t>
+          <t>but the US lane is viable, which it was not before the retention correction below.</t>
         </is>
       </c>
     </row>
@@ -799,28 +805,35 @@
     <row r="34">
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>dominate. Repeat rate still governs long-run value and every year after year two —</t>
+          <t>RETENTION CORRECTION — 2 Sep 2026</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>track it — but do not let it decide the supplier. The supplier quote decides payback.</t>
+          <t>This model originally assumed 0.78 monthly retention, implying ~5% of repeat</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>customers survive a year. Published pet-subscription benchmarks put retention at</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>CONSEQUENCE: the US lane only works if a real quote beats these placeholders —</t>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>60%+ past month 12. Corrected to 0.990 (quarterly billing). Effect: 24-month</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>roughly FOB at or below $5.00, or MOQ at or below 1,500. Ask for both in the RFQ.</t>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>EBITDA roughly doubles, PHP 3.6M to PHP 6.7M, and payback moves 15 to 13 months.</t>
         </is>
       </c>
     </row>
@@ -828,6 +841,49 @@
       <c r="B39" s="4" t="inlineStr">
         <is>
           <t>Note too that US-lane wholesale margin lands at ~29%, just under the 30% screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="46" t="inlineStr">
+        <is>
+          <t>CONSEQUENCE FOR REPEAT RATE: with retention corrected, repeat customers are ~72%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="46" t="inlineStr">
+        <is>
+          <t>of month-24 volume. Repeat conversion from 10% to 45% swings 24-month EBITDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="46" t="inlineStr">
+        <is>
+          <t>2.4x (PHP 3.3M to 8.1M) while moving payback only 16 to 13 months. So repeat rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="46" t="inlineStr">
+        <is>
+          <t>sets what the business earns and is worth; landed cost sets when it pays back.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44"/>
+    <row r="45">
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Sell QUARTERLY by default. Benchmarks: monthly plans churn 18-22%/yr, quarterly</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>11-16%/yr, and longer billing cadence cuts churn without raising acquisition cost.</t>
         </is>
       </c>
     </row>
@@ -1138,11 +1194,11 @@
         </is>
       </c>
       <c r="C27" s="14" t="n">
-        <v>0.78</v>
+        <v>0.99</v>
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Quarterly billing. Use 0.982 if billing monthly.</t>
         </is>
       </c>
     </row>
@@ -1173,6 +1229,13 @@
       <c r="D29" s="10" t="inlineStr">
         <is>
           <t>1.0 = base. Scenarios tab uses 0.6 / 1.0 / 1.5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Billing cadence note: quarterly billing cuts churn without raising CAC.</t>
         </is>
       </c>
     </row>

</xml_diff>